<commit_message>
PMBIPO-324 - Update production dataset fixtures
</commit_message>
<xml_diff>
--- a/api/src/portal/db/init/data/errors/rejected_rows.xlsx
+++ b/api/src/portal/db/init/data/errors/rejected_rows.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="53">
   <si>
     <t>Function</t>
   </si>
@@ -22,12 +22,18 @@
     <t>SubFunction</t>
   </si>
   <si>
+    <t>Group</t>
+  </si>
+  <si>
     <t>Site</t>
   </si>
   <si>
     <t>Display Name</t>
   </si>
   <si>
+    <t>Data Source(s)</t>
+  </si>
+  <si>
     <t>Category</t>
   </si>
   <si>
@@ -58,64 +64,112 @@
     <t>Restricted</t>
   </si>
   <si>
+    <t>Finance</t>
+  </si>
+  <si>
+    <t>Human Resources</t>
+  </si>
+  <si>
     <t>Operations</t>
   </si>
   <si>
-    <t>Finance</t>
-  </si>
-  <si>
-    <t>Quality</t>
+    <t>Program Management</t>
+  </si>
+  <si>
+    <t>General::Finance</t>
+  </si>
+  <si>
+    <t>General::Human Resources</t>
   </si>
   <si>
     <t>General::Operations</t>
   </si>
   <si>
-    <t>Program Finance</t>
-  </si>
-  <si>
-    <t>SAS Operations Scorecard</t>
+    <t>e3</t>
+  </si>
+  <si>
+    <t>General::Program Management</t>
+  </si>
+  <si>
+    <t>Adoption Metrics</t>
+  </si>
+  <si>
+    <t>PLT Certification Dashboards</t>
+  </si>
+  <si>
+    <t>SAS Segment e3 Site</t>
+  </si>
+  <si>
+    <t>Program Health Dashboard</t>
   </si>
   <si>
     <t>Cobra Standardization</t>
   </si>
   <si>
-    <t>Program Health Dashboard (PHD)</t>
+    <t>PeopleSoft, Success Factors, StaffIt</t>
+  </si>
+  <si>
+    <t>SharePoint</t>
+  </si>
+  <si>
+    <t>PeopleSoft, HypFcst, Cobra</t>
+  </si>
+  <si>
+    <t>Cobra</t>
   </si>
   <si>
     <t>tableau</t>
   </si>
   <si>
-    <t>The SAS Operations Scorecard pulls monthly Tier 1 EHS, Production, Quality, and Supply Chain metrics from Athena for Monthly Operating Reviews (MOR).</t>
-  </si>
-  <si>
-    <t>Highlights required fields in Cobra and tracks the status for each program.</t>
+    <t>sharepoint</t>
+  </si>
+  <si>
+    <t>Program Management Training and Certifications dashboards.</t>
+  </si>
+  <si>
+    <t>e3 resource support site specific to the SAS segment. This site includes communications, metrics, training details, and best practices for teams to be able to leverage to achieve e3 objectives.</t>
   </si>
   <si>
     <t>The Program Health Dashboard offers metrics relevant to Program performance over the past 12 periods. Includes Contract Information, Financial Summary, and Earned Value metrics.</t>
   </si>
   <si>
-    <t>https://tableau.l3harris.com/#/workbooks/4973/views</t>
+    <t>Outlines standard data fields required in Cobra and tracks the status of adoption for each program.</t>
+  </si>
+  <si>
+    <t>https://tableau.l3harris.com/#/workbooks/10943/views</t>
+  </si>
+  <si>
+    <t>https://l3t.sharepoint.us/sites/SASOperationalExcellence</t>
+  </si>
+  <si>
+    <t>https://tableau.l3harris.com/#/workbooks/9049/views</t>
   </si>
   <si>
     <t>https://tableau.l3harris.com/#/workbooks/9489/views</t>
   </si>
   <si>
-    <t>https://tableau.l3harris.com/#/workbooks/9049/views</t>
-  </si>
-  <si>
-    <t>meghan.mcmorrow@harris.com</t>
+    <t>jim.behnke@harris.com</t>
+  </si>
+  <si>
+    <t>jack.riesen@harris.com</t>
+  </si>
+  <si>
+    <t>melissa.cataldo@harris.com</t>
   </si>
   <si>
     <t>cyle.powers@harris.com</t>
   </si>
   <si>
-    <t>sandra.williams@harris.com</t>
-  </si>
-  <si>
-    <t>Operations, Scorecard, Athena</t>
-  </si>
-  <si>
-    <t>PHD, Earned Value, Program Performance</t>
+    <t>david.sandor@harris.com</t>
+  </si>
+  <si>
+    <t>Certifications, PLT, IPTL, CAM, Training Requirements, Program Leadership</t>
+  </si>
+  <si>
+    <t>Earned Value, EVMS, Program Finance, PHD, Program Performance</t>
+  </si>
+  <si>
+    <t>Data Standards, Earned Value, EVMS</t>
   </si>
   <si>
     <t>X</t>
@@ -489,10 +543,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:Q8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:15">
+    <row r="1" spans="1:17">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -535,147 +589,321 @@
       <c r="O1" s="1" t="s">
         <v>13</v>
       </c>
+      <c r="P1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>15</v>
+      </c>
     </row>
-    <row r="2" spans="1:15">
+    <row r="2" spans="1:17">
       <c r="A2" s="1">
-        <v>133</v>
+        <v>58</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H2" t="s">
+        <v>34</v>
+      </c>
+      <c r="I2" t="s">
+        <v>36</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="K2" t="s">
+        <v>44</v>
+      </c>
+      <c r="L2" t="s">
+        <v>48</v>
+      </c>
+      <c r="M2" t="s">
+        <v>49</v>
+      </c>
+      <c r="N2" t="s">
+        <v>52</v>
+      </c>
+      <c r="O2" t="s">
+        <v>52</v>
+      </c>
+      <c r="P2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17">
+      <c r="A3" s="1">
+        <v>85</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G3" t="s">
+        <v>30</v>
+      </c>
+      <c r="H3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I3" t="s">
+        <v>36</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="K3" t="s">
+        <v>44</v>
+      </c>
+      <c r="L3" t="s">
+        <v>48</v>
+      </c>
+      <c r="M3" t="s">
+        <v>49</v>
+      </c>
+      <c r="N3" t="s">
+        <v>52</v>
+      </c>
+      <c r="O3" t="s">
+        <v>52</v>
+      </c>
+      <c r="P3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17">
+      <c r="A4" s="1">
+        <v>118</v>
+      </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I4" t="s">
+        <v>36</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="K4" t="s">
+        <v>44</v>
+      </c>
+      <c r="L4" t="s">
+        <v>48</v>
+      </c>
+      <c r="M4" t="s">
+        <v>49</v>
+      </c>
+      <c r="N4" t="s">
+        <v>52</v>
+      </c>
+      <c r="O4" t="s">
+        <v>52</v>
+      </c>
+      <c r="P4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17">
+      <c r="A5" s="1">
+        <v>119</v>
+      </c>
+      <c r="B5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F5" t="s">
+        <v>27</v>
+      </c>
+      <c r="G5" t="s">
+        <v>31</v>
+      </c>
+      <c r="H5" t="s">
+        <v>35</v>
+      </c>
+      <c r="I5" t="s">
+        <v>37</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="K5" t="s">
+        <v>45</v>
+      </c>
+      <c r="L5" t="s">
+        <v>45</v>
+      </c>
+      <c r="M5" t="s">
+        <v>23</v>
+      </c>
+      <c r="N5" t="s">
+        <v>52</v>
+      </c>
+      <c r="O5" t="s">
+        <v>52</v>
+      </c>
+      <c r="P5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17">
+      <c r="A6" s="1">
+        <v>120</v>
+      </c>
+      <c r="B6" t="s">
         <v>19</v>
       </c>
-      <c r="F2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G2" t="s">
-        <v>23</v>
-      </c>
-      <c r="H2" s="2" t="s">
+      <c r="C6" t="s">
+        <v>24</v>
+      </c>
+      <c r="F6" t="s">
+        <v>28</v>
+      </c>
+      <c r="G6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H6" t="s">
+        <v>34</v>
+      </c>
+      <c r="I6" t="s">
+        <v>38</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="K6" t="s">
+        <v>46</v>
+      </c>
+      <c r="M6" t="s">
+        <v>50</v>
+      </c>
+      <c r="N6" t="s">
+        <v>52</v>
+      </c>
+      <c r="O6" t="s">
+        <v>52</v>
+      </c>
+      <c r="P6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17">
+      <c r="A7" s="1">
+        <v>122</v>
+      </c>
+      <c r="B7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" t="s">
+        <v>25</v>
+      </c>
+      <c r="F7" t="s">
+        <v>29</v>
+      </c>
+      <c r="G7" t="s">
+        <v>33</v>
+      </c>
+      <c r="H7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I7" t="s">
+        <v>39</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="K7" t="s">
+        <v>47</v>
+      </c>
+      <c r="M7" t="s">
+        <v>51</v>
+      </c>
+      <c r="N7" t="s">
+        <v>52</v>
+      </c>
+      <c r="O7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17">
+      <c r="A8" s="1">
+        <v>134</v>
+      </c>
+      <c r="B8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" t="s">
+        <v>24</v>
+      </c>
+      <c r="F8" t="s">
         <v>26</v>
       </c>
-      <c r="I2" t="s">
-        <v>29</v>
-      </c>
-      <c r="K2" t="s">
-        <v>32</v>
-      </c>
-      <c r="N2" t="s">
+      <c r="G8" t="s">
+        <v>30</v>
+      </c>
+      <c r="H8" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="3" spans="1:15">
-      <c r="A3" s="1">
-        <v>157</v>
-      </c>
-      <c r="B3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F3" t="s">
-        <v>22</v>
-      </c>
-      <c r="G3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="I3" t="s">
-        <v>29</v>
-      </c>
-      <c r="K3" t="s">
-        <v>32</v>
-      </c>
-      <c r="N3" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15">
-      <c r="A4" s="1">
-        <v>211</v>
-      </c>
-      <c r="B4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" t="s">
-        <v>22</v>
-      </c>
-      <c r="G4" t="s">
-        <v>24</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="I4" t="s">
-        <v>30</v>
-      </c>
-      <c r="L4" t="s">
-        <v>34</v>
-      </c>
-      <c r="M4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15">
-      <c r="A5" s="1">
-        <v>212</v>
-      </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" t="s">
-        <v>21</v>
-      </c>
-      <c r="F5" t="s">
-        <v>22</v>
-      </c>
-      <c r="G5" t="s">
-        <v>25</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="I5" t="s">
-        <v>31</v>
-      </c>
-      <c r="K5" t="s">
-        <v>33</v>
-      </c>
-      <c r="L5" t="s">
-        <v>34</v>
-      </c>
-      <c r="M5" t="s">
-        <v>34</v>
-      </c>
-      <c r="N5" t="s">
-        <v>34</v>
+      <c r="I8" t="s">
+        <v>36</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="K8" t="s">
+        <v>44</v>
+      </c>
+      <c r="L8" t="s">
+        <v>48</v>
+      </c>
+      <c r="M8" t="s">
+        <v>49</v>
+      </c>
+      <c r="N8" t="s">
+        <v>52</v>
+      </c>
+      <c r="O8" t="s">
+        <v>52</v>
+      </c>
+      <c r="P8" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="H2" r:id="rId1" location="/workbooks/4973/views"/>
-    <hyperlink ref="H3" r:id="rId2" location="/workbooks/4973/views"/>
-    <hyperlink ref="H4" r:id="rId3" location="/workbooks/9489/views"/>
-    <hyperlink ref="H5" r:id="rId4" location="/workbooks/9049/views"/>
+    <hyperlink ref="J2" r:id="rId1" location="/workbooks/10943/views"/>
+    <hyperlink ref="J3" r:id="rId2" location="/workbooks/10943/views"/>
+    <hyperlink ref="J4" r:id="rId3" location="/workbooks/10943/views"/>
+    <hyperlink ref="J5" r:id="rId4"/>
+    <hyperlink ref="J6" r:id="rId5" location="/workbooks/9049/views"/>
+    <hyperlink ref="J7" r:id="rId6" location="/workbooks/9489/views"/>
+    <hyperlink ref="J8" r:id="rId7" location="/workbooks/10943/views"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
PMBIPO-324 - Update production data with missing manufacturing&quality function, quality subfunction
</commit_message>
<xml_diff>
--- a/api/src/portal/db/init/data/errors/rejected_rows.xlsx
+++ b/api/src/portal/db/init/data/errors/rejected_rows.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="59">
   <si>
     <t>Function</t>
   </si>
@@ -97,6 +97,9 @@
     <t>PLT Certification Dashboards</t>
   </si>
   <si>
+    <t>SAS Operations Scorecard</t>
+  </si>
+  <si>
     <t>SAS Segment e3 Site</t>
   </si>
   <si>
@@ -109,6 +112,9 @@
     <t>PeopleSoft, Success Factors, StaffIt</t>
   </si>
   <si>
+    <t>Athena, Gensuite</t>
+  </si>
+  <si>
     <t>SharePoint</t>
   </si>
   <si>
@@ -127,6 +133,9 @@
     <t>Program Management Training and Certifications dashboards.</t>
   </si>
   <si>
+    <t>The SAS Operations Scorecard pulls monthly Tier 1 EHS, Production, Quality, and Supply Chain metrics from Athena for Monthly Operating Reviews (MOR).</t>
+  </si>
+  <si>
     <t>e3 resource support site specific to the SAS segment. This site includes communications, metrics, training details, and best practices for teams to be able to leverage to achieve e3 objectives.</t>
   </si>
   <si>
@@ -139,6 +148,9 @@
     <t>https://tableau.l3harris.com/#/workbooks/10943/views</t>
   </si>
   <si>
+    <t>https://tableau.l3harris.com/#/workbooks/4973/views</t>
+  </si>
+  <si>
     <t>https://l3t.sharepoint.us/sites/SASOperationalExcellence</t>
   </si>
   <si>
@@ -151,6 +163,9 @@
     <t>jim.behnke@harris.com</t>
   </si>
   <si>
+    <t>meghan.mcmorrow@harris.com</t>
+  </si>
+  <si>
     <t>jack.riesen@harris.com</t>
   </si>
   <si>
@@ -164,6 +179,9 @@
   </si>
   <si>
     <t>Certifications, PLT, IPTL, CAM, Training Requirements, Program Leadership</t>
+  </si>
+  <si>
+    <t>Operations, Scorecard, Athena</t>
   </si>
   <si>
     <t>Earned Value, EVMS, Program Finance, PHD, Program Performance</t>
@@ -543,7 +561,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q8"/>
+  <dimension ref="A1:Q9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
@@ -610,34 +628,34 @@
         <v>26</v>
       </c>
       <c r="G2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="K2" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="L2" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="M2" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="N2" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="O2" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="P2" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -654,39 +672,39 @@
         <v>26</v>
       </c>
       <c r="G3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="K3" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="L3" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="M3" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="N3" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="O3" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="P3" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:17">
       <c r="A4" s="1">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="B4" t="s">
         <v>18</v>
@@ -695,215 +713,251 @@
         <v>22</v>
       </c>
       <c r="F4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G4" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="H4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I4" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="K4" t="s">
-        <v>44</v>
-      </c>
-      <c r="L4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="M4" t="s">
-        <v>49</v>
-      </c>
-      <c r="N4" t="s">
-        <v>52</v>
-      </c>
-      <c r="O4" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="P4" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:17">
       <c r="A5" s="1">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="B5" t="s">
         <v>18</v>
       </c>
       <c r="C5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G5" t="s">
         <v>31</v>
       </c>
       <c r="H5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="I5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="K5" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="L5" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="M5" t="s">
-        <v>23</v>
+        <v>54</v>
       </c>
       <c r="N5" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="O5" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="P5" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:17">
       <c r="A6" s="1">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F6" t="s">
         <v>28</v>
       </c>
       <c r="G6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H6" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="I6" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K6" t="s">
-        <v>46</v>
+        <v>50</v>
+      </c>
+      <c r="L6" t="s">
+        <v>50</v>
       </c>
       <c r="M6" t="s">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="N6" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="O6" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="P6" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
     </row>
     <row r="7" spans="1:17">
       <c r="A7" s="1">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="B7" t="s">
         <v>19</v>
       </c>
       <c r="C7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F7" t="s">
         <v>29</v>
       </c>
       <c r="G7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I7" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="K7" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="M7" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="N7" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="O7" t="s">
-        <v>52</v>
+        <v>58</v>
+      </c>
+      <c r="P7" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="8" spans="1:17">
       <c r="A8" s="1">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B8" t="s">
         <v>19</v>
       </c>
       <c r="C8" t="s">
+        <v>25</v>
+      </c>
+      <c r="F8" t="s">
+        <v>30</v>
+      </c>
+      <c r="G8" t="s">
+        <v>35</v>
+      </c>
+      <c r="H8" t="s">
+        <v>36</v>
+      </c>
+      <c r="I8" t="s">
+        <v>42</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="K8" t="s">
+        <v>52</v>
+      </c>
+      <c r="M8" t="s">
+        <v>57</v>
+      </c>
+      <c r="N8" t="s">
+        <v>58</v>
+      </c>
+      <c r="O8" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17">
+      <c r="A9" s="1">
+        <v>143</v>
+      </c>
+      <c r="B9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" t="s">
         <v>24</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F9" t="s">
         <v>26</v>
       </c>
-      <c r="G8" t="s">
-        <v>30</v>
-      </c>
-      <c r="H8" t="s">
-        <v>34</v>
-      </c>
-      <c r="I8" t="s">
+      <c r="G9" t="s">
+        <v>31</v>
+      </c>
+      <c r="H9" t="s">
         <v>36</v>
       </c>
-      <c r="J8" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="K8" t="s">
-        <v>44</v>
-      </c>
-      <c r="L8" t="s">
+      <c r="I9" t="s">
+        <v>38</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="K9" t="s">
         <v>48</v>
       </c>
-      <c r="M8" t="s">
-        <v>49</v>
-      </c>
-      <c r="N8" t="s">
-        <v>52</v>
-      </c>
-      <c r="O8" t="s">
-        <v>52</v>
-      </c>
-      <c r="P8" t="s">
-        <v>52</v>
+      <c r="L9" t="s">
+        <v>53</v>
+      </c>
+      <c r="M9" t="s">
+        <v>54</v>
+      </c>
+      <c r="N9" t="s">
+        <v>58</v>
+      </c>
+      <c r="O9" t="s">
+        <v>58</v>
+      </c>
+      <c r="P9" t="s">
+        <v>58</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="J2" r:id="rId1" location="/workbooks/10943/views"/>
     <hyperlink ref="J3" r:id="rId2" location="/workbooks/10943/views"/>
-    <hyperlink ref="J4" r:id="rId3" location="/workbooks/10943/views"/>
-    <hyperlink ref="J5" r:id="rId4"/>
-    <hyperlink ref="J6" r:id="rId5" location="/workbooks/9049/views"/>
-    <hyperlink ref="J7" r:id="rId6" location="/workbooks/9489/views"/>
-    <hyperlink ref="J8" r:id="rId7" location="/workbooks/10943/views"/>
+    <hyperlink ref="J4" r:id="rId3" location="/workbooks/4973/views"/>
+    <hyperlink ref="J5" r:id="rId4" location="/workbooks/10943/views"/>
+    <hyperlink ref="J6" r:id="rId5"/>
+    <hyperlink ref="J7" r:id="rId6" location="/workbooks/9049/views"/>
+    <hyperlink ref="J8" r:id="rId7" location="/workbooks/9489/views"/>
+    <hyperlink ref="J9" r:id="rId8" location="/workbooks/10943/views"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>